<commit_message>
update excel addin link
</commit_message>
<xml_diff>
--- a/source/_static/sample-award-12.xlsx
+++ b/source/_static/sample-award-12.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15160"/>
+    <workbookView windowHeight="15360"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Compitition</t>
+    <t>Competition</t>
   </si>
   <si>
     <t>Award</t>

</xml_diff>